<commit_message>
Added test cases and some documentation side-slide content
</commit_message>
<xml_diff>
--- a/tests/bpDashboardTestSuite.xlsx
+++ b/tests/bpDashboardTestSuite.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29825"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29910"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{02DA46BA-4636-4D38-9A5E-C742705FF284}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{EC07EF1F-A64B-46DA-B55B-4D6C1C5C053C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" firstSheet="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" firstSheet="3" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="DashboardTestPlan" sheetId="1" r:id="rId1"/>
@@ -13,11 +13,9 @@
     <sheet name="AppsScriptTestPlan" sheetId="6" r:id="rId3"/>
     <sheet name="Documentation" sheetId="3" r:id="rId4"/>
     <sheet name="TestSummary" sheetId="4" r:id="rId5"/>
-    <sheet name="Open a defect." sheetId="5" r:id="rId6"/>
-    <sheet name="IsADefect" sheetId="7" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">DashboardTestPlan!$A$1:$P$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">DashboardTestPlan!$A$1:$O$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">AppsScriptTestPlan!$A$1:$O$1</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
@@ -43,19 +41,10 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
-    <author>tc={0AB13653-40C4-47FA-A319-C6506C77DB43}</author>
     <author>tc={B2C5348B-3D7D-45CA-ACA4-7E3CA42663CE}</author>
   </authors>
   <commentList>
-    <comment ref="E1" authorId="0" shapeId="0" xr:uid="{0AB13653-40C4-47FA-A319-C6506C77DB43}">
-      <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-    gemini suggested keeping the same depth - not only for pivot tables, but it makes your GitHub repo look like it was designed by someone who knows how to architect a test suite, not just list tasks.</t>
-      </text>
-    </comment>
-    <comment ref="F1" authorId="1" shapeId="0" xr:uid="{B2C5348B-3D7D-45CA-ACA4-7E3CA42663CE}">
+    <comment ref="E1" authorId="0" shapeId="0" xr:uid="{B2C5348B-3D7D-45CA-ACA4-7E3CA42663CE}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -95,7 +84,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="377" uniqueCount="263">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="421" uniqueCount="240">
   <si>
     <t>Priority</t>
   </si>
@@ -127,27 +116,6 @@
     </r>
   </si>
   <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>OLD</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> Subject (Folder) Path String</t>
-    </r>
-  </si>
-  <si>
     <t>Description</t>
   </si>
   <si>
@@ -193,10 +161,7 @@
     <t>UI/User Agent</t>
   </si>
   <si>
-    <t>Application/UI/IOS/Safari</t>
-  </si>
-  <si>
-    <t>.css block z-index order.</t>
+    <t>Verify page &lt;divs&gt;/&lt;sections&gt;  render sanely according do z-index (e.g. header should not draw on top of error banner, obscuring it)</t>
   </si>
   <si>
     <t>TC-01</t>
@@ -219,9 +184,6 @@
     <t>Passed</t>
   </si>
   <si>
-    <t>Application/UI/OS X/Safari</t>
-  </si>
-  <si>
     <t>TC-02</t>
   </si>
   <si>
@@ -231,25 +193,19 @@
     <t>Blocked</t>
   </si>
   <si>
-    <t>Application/UI/Windows/Chrome</t>
-  </si>
-  <si>
     <t>TC-03</t>
   </si>
   <si>
     <t>Windows/Chrome .css layer order</t>
   </si>
   <si>
-    <t>Application/UI/Android/Chrome</t>
-  </si>
-  <si>
     <t>TC-04</t>
   </si>
   <si>
     <t>Android/Chrome .css layer order</t>
   </si>
   <si>
-    <t>Low</t>
+    <t>High</t>
   </si>
   <si>
     <t>Javascript is disabled in a browser
@@ -272,10 +228,10 @@
     <t>&lt;noscript&gt; message executes and the plain html and .css renders.</t>
   </si>
   <si>
+    <t>Low</t>
+  </si>
+  <si>
     <t>UI/Functional/State</t>
-  </si>
-  <si>
-    <t>Application/UI/Async Checks</t>
   </si>
   <si>
     <t>Typical design where an application is pulling from an api in async/await action.</t>
@@ -294,7 +250,7 @@
     <t>Overaly appears, spinner rotates.</t>
   </si>
   <si>
-    <t>???</t>
+    <t>Design</t>
   </si>
   <si>
     <t>Gemini said I already handled a scenario if the json is ready before the DOM is fully loaded.  Where's the code, what's the test called, and what are the steps?</t>
@@ -312,47 +268,67 @@
     <t>Verify system generates a UI banner if the user is attempting to view data from a malformed .json data source, causing the whole parser to panic and whole file to fail.</t>
   </si>
   <si>
-    <t>User is warned if data source has fatal syntax error.</t>
+    <t>Log is generated if application data source contains a fatal syntax error.</t>
+  </si>
+  <si>
+    <t>Pick a syntax rule...any rule, and break it.</t>
   </si>
   <si>
     <t>Synthesize a malformed record where the application retrieves data from:
-- try "Sys": , in the json response file.
-Hard reload page and observe browser.</t>
-  </si>
-  <si>
-    <t>Banner is displayed with a warning message.</t>
+- Remove a Sys key value pair from bp_readings.json
+- Hard reload page and observe UI.</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Banner is displayed with a warning message. &lt;- </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>What message?</t>
+    </r>
   </si>
   <si>
     <t>Passes, however a code change is needed - opened Issue # 39</t>
   </si>
   <si>
-    <t>Application/Dependencies</t>
-  </si>
-  <si>
-    <t>The UI test is for humans hitting the page - that includes HEADLESS selenium, google/bing bots &amp; playwrite which execute javascript.
-This test is for FB&amp;X crawlers/AI LLMs/Lynx/Discord/paranoid chrome&amp;firefox users.
-- Can console.log test w/ selenium so automate on &lt;noscript&gt; element - see documentation.</t>
-  </si>
-  <si>
-    <t>TC 01</t>
-  </si>
-  <si>
-    <t>Execute automation test.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Application/Dependencies </t>
-  </si>
-  <si>
-    <t>font handling: remove google font &lt;link rel="..."&gt; tags</t>
-  </si>
-  <si>
-    <t>&lt;- this is an application dependency, and not a "UI/" folder - I only verify in the UI. I will check the browser safe fonts, but also the code changes needed for github issue #14 for retina and device pixel ratios</t>
-  </si>
-  <si>
-    <t>chart.js handling: remove CDN &lt;script src="..."&gt; tags 1 by 1.</t>
-  </si>
-  <si>
-    <t>&lt;- gemini said something about a failover test?  Failover at CDN or on my end?</t>
+    <t>The data source or file is simply not reachable.</t>
+  </si>
+  <si>
+    <t>Log is generated if application data source is missing.</t>
+  </si>
+  <si>
+    <t>Missing data.json file</t>
+  </si>
+  <si>
+    <t>Rename or delete bp_readings.json
+Load dashboard and observe UI.</t>
+  </si>
+  <si>
+    <t>Error banner should trigger with "404: Failed To Load Data" message</t>
+  </si>
+  <si>
+    <t>The data source returns something, but it is an empty array containing 0 records.</t>
+  </si>
+  <si>
+    <t>Log is generated if application data source is incomplete.</t>
+  </si>
+  <si>
+    <t>Empty data.json array</t>
+  </si>
+  <si>
+    <t>delete all data within .json, leaving "[]" object.
+Load dashboard and observe UI</t>
   </si>
   <si>
     <r>
@@ -362,8 +338,7 @@
         <rFont val="Calibri"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve">How do chart modules react?
-</t>
+      <t xml:space="preserve">Banner is displayed with a warning message. </t>
     </r>
     <r>
       <rPr>
@@ -372,51 +347,8 @@
         <rFont val="Calibri"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve">- errorhandling.js has checkChartDependencies() that should show a warning in each module - does it work??
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">How does error banner react?
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">checkChartDependencies() should throw an error banner too - does it work??
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">How do console logs react?
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>checkChartDependencies() does log with a testable message.  Does it work?</t>
-    </r>
-  </si>
-  <si>
-    <t>Application/Errors/Module isolation</t>
+      <t>&lt;- What message?</t>
+    </r>
   </si>
   <si>
     <r>
@@ -449,54 +381,245 @@
 How does the console log react?</t>
   </si>
   <si>
-    <t>Application/Errors/Error Handling</t>
+    <t>UI/Functional/Reporting</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Write these - start with reconciliation.  This is not console testing; this is the new &lt;div&gt; module I need to design into the dashboard.  
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>There's at least 1 defect - I removed a value from a Key (therefore it's null) and the record was dropped as confirmed by Raw Data Table chart, but the "[NORMALIZER] Successfully normalized:  Records: nnn" did not decrement that dropped record &lt;- That's an automation application/data integrity test though.</t>
+    </r>
+  </si>
+  <si>
+    <t>UI/Functional/Cross Chart verification</t>
+  </si>
+  <si>
+    <t>Verify Last Reading Date; MAX(Date)</t>
+  </si>
+  <si>
+    <t>Verify Last Reading Date is consistent across charts</t>
+  </si>
+  <si>
+    <t>ETL from gSheet runs, data.json loaded successfully.</t>
+  </si>
+  <si>
+    <t>Open dashboard, check raw table, check header, check .json</t>
+  </si>
+  <si>
+    <t>Last Reading Date in header matches latest reading date in Raw table, matches latest .json record</t>
+  </si>
+  <si>
+    <t>Header value is "reading date unavailable" on load but has a value after reloading the page.</t>
+  </si>
+  <si>
+    <t>Failed</t>
+  </si>
+  <si>
+    <t>Open a defect.</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Verify Averages.  </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>This is tricky - I made a conscious decision and wrote it down somewhere that averages didn't have to match up - where did I write that down?</t>
+    </r>
+  </si>
+  <si>
+    <t>Verify Averages are consistent across charts</t>
+  </si>
+  <si>
+    <t>UI/Functional/Formatting</t>
+  </si>
+  <si>
+    <t>These are module UI checks because the source has datetime and the x-axis shows different formats, while tooltips show hh-mm-ssAMPM ONLY if it's not an Avg() type chart.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verify special datetime formatting matches record </t>
+  </si>
+  <si>
+    <t>Application/Dependencies</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">The UI test is for humans hitting the page - that includes HEADLESS selenium, google/bing bots &amp; playwrite which execute javascript.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">This test </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>is for FB&amp;X crawlers/AI LLMs/Lynx/Discord/paranoid chrome&amp;firefox users.
+- Can console.log test w/ selenium so automate on &lt;noscript&gt; element - see documentation.</t>
+    </r>
+  </si>
+  <si>
+    <t>Execute automation test.</t>
+  </si>
+  <si>
+    <t>font handling: remove google font &lt;link rel="..."&gt; tags</t>
+  </si>
+  <si>
+    <t>&lt;- this is an application dependency, and not a "UI/" folder - I only verify in the UI. I will check the browser safe fonts, but also the code changes needed for github issue #14 for retina and device pixel ratios</t>
+  </si>
+  <si>
+    <t>chart.js handling: remove CDN &lt;script src="..."&gt; tags 1 by 1.</t>
+  </si>
+  <si>
+    <t>&lt;- gemini said something about a failover test?  Failover at CDN or on my end?</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">How do chart modules react?
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">- errorhandling.js has checkChartDependencies() that should show a warning in each module - does it work??
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">How does error banner react?
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">checkChartDependencies() should throw an error banner too - does it work??
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">How do console logs react?
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>checkChartDependencies() does log with a testable message.  Does it work?</t>
+    </r>
+  </si>
+  <si>
+    <t>Application/Error Handling</t>
   </si>
   <si>
     <t>&lt;- deconstruct utils/errorhandling.js for cases</t>
   </si>
   <si>
-    <t>Application/Error Handling</t>
-  </si>
-  <si>
     <t>How does AbortController() currently in use work regarding timeouts?  Does it console.warn and should it errorbanner the user?</t>
   </si>
   <si>
-    <t>Verify a log is generated if  the application processes a .json data source, causing the whole parser to panic and whole file to fail.</t>
-  </si>
-  <si>
-    <t>Log is generated if data source has fatal syntax error.</t>
+    <t>Verify a log is generated if  the application processes a .json data source, causing the parser to panic and whole file to fail.</t>
   </si>
   <si>
     <t>Synthesize a malformed record where the application retrieves data from:
-- try "Sys": , in the json response file.
-Hard reload page and observe console.</t>
-  </si>
-  <si>
-    <t>UI shows "Failed to Load Data" banner; 
-Console logs SyntaxError.</t>
-  </si>
-  <si>
-    <t>Log is generated.</t>
-  </si>
-  <si>
-    <t>Application/Data/Error Handling</t>
-  </si>
-  <si>
-    <t>Missing data.json file</t>
+- Remove a Sys key value pair from bp_readings.json
+- Hard reload page and observe console.</t>
+  </si>
+  <si>
+    <t>Console logs SyntaxError. &lt;- What is the message?</t>
+  </si>
+  <si>
+    <t>"Rename or delete bp_readings.json
+Load dashboard.</t>
+  </si>
+  <si>
+    <t>Console logs "DATA LOADER] ❌ Failed to load data: Error: HTTP 404"</t>
+  </si>
+  <si>
+    <t>Log is generated</t>
+  </si>
+  <si>
+    <t>Automated</t>
+  </si>
+  <si>
+    <t>Empty data.json file</t>
   </si>
   <si>
     <t>delete all data within .json.
 Load dashboard</t>
   </si>
   <si>
-    <t>How do chart modules react?
-How does error banner react?
-How do console logs react?</t>
-  </si>
-  <si>
-    <t>Empty data.json file</t>
-  </si>
-  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">How do console logs react?
+bp_data_loader.js should console.log a "Data array is empty" entry. </t>
+    </r>
     <r>
       <rPr>
         <sz val="11"/>
@@ -504,95 +627,104 @@
         <rFont val="Calibri"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve">How do chart modules react?
-How does error banner react?
-How do console logs react?
-Scenario: GitHub serves a file that is just [] (an empty array).
-Expected Result: bp_data_loader.js should throw the error "Data array is empty" and trigger the showErrorState UI.  </t>
-    </r>
+      <t>&lt;- What is the exact message?</t>
+    </r>
+  </si>
+  <si>
+    <t>Application/Data Integrity</t>
+  </si>
+  <si>
     <r>
       <rPr>
         <b/>
         <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">&lt;- this is huge - this category will discuss all the "cleaning" or "shaping' of data like converting "120" to 120 - It’s the process of taking "messy" data (like dates in different formats or numbers as strings) and making them all look the same so your charts don't break. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
         <color rgb="FFFF0000"/>
         <rFont val="Calibri"/>
         <scheme val="minor"/>
       </rPr>
-      <t>Does it?  Does it console.log for testing??</t>
-    </r>
-  </si>
-  <si>
-    <t>Application/Data/Data Integrity</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
+      <t>Already started below...need to add more of those tests, and also reproduce it up in the UI/Reporting set.</t>
+    </r>
+  </si>
+  <si>
+    <t>add a pivot table or something foreign in the gSheet sheet</t>
+  </si>
+  <si>
+    <t>&lt;- remember how Tableau failed?  What should I look for in my  application without a schema validation?  I know json is "take what you need and ignore the rest, but what could cause it to catastrophically fail?</t>
+  </si>
+  <si>
+    <t>add data with empty required fields</t>
+  </si>
+  <si>
+    <t>add string in integer field</t>
+  </si>
+  <si>
+    <t>&lt;- There is code for this - gemini showed where but I didn't see it - I should make a console log and test for it.</t>
+  </si>
+  <si>
+    <t>add formula (like an accidental reference) in integer field</t>
+  </si>
+  <si>
+    <t>&lt;- This could happen at source and here as well - both need attention.</t>
+  </si>
+  <si>
+    <t>Fault, not failure - Dia key has Sys value</t>
+  </si>
+  <si>
+    <t>&lt;- Is there any way I can determine if Dia data comes in labeled Sys and vice versa by accident?   They're both 2 digit numbers.</t>
+  </si>
+  <si>
+    <t>???</t>
+  </si>
+  <si>
+    <t>&lt;- I check for strings in int fields, but not dates in int fields, do I? I don't have field value requirements written, like int(2) or float(), or string(len) for Comments.</t>
+  </si>
+  <si>
+    <t>Reject future dates.</t>
+  </si>
+  <si>
+    <t>Need validation code - I don't specifically look for it now so these will sneak in currently.</t>
+  </si>
+  <si>
+    <t>Reject dates older than (60?) years</t>
+  </si>
+  <si>
+    <t>Reject "0" value records</t>
+  </si>
+  <si>
+    <t>currently validateNumericReading checks for min: 40 so 0 would be dropped - is that true?  I didn't write a requirement for this!</t>
+  </si>
+  <si>
+    <t>Handle Leap Years</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
         <rFont val="Calibri"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve">&lt;- this is huge - this category will discuss all the "cleaning" or "shaping' of data like converting "120" to 120 - It’s the process of taking "messy" data (like dates in different formats or numbers as strings) and making them all look the same so your charts don't break. </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
+      <t xml:space="preserve">&lt;- Gemini said something about me not rejecting a record if Feb 29 shows up on a non-leap year but instead map() moves it to March 1st.  </t>
+    </r>
+    <r>
+      <rPr>
         <sz val="11"/>
         <color rgb="FFFF0000"/>
         <rFont val="Calibri"/>
         <scheme val="minor"/>
       </rPr>
-      <t>Already started below...need to add more of those tests. Gemini said I drop nulls and there's a defect for Sys&lt;=40 being dropped.</t>
-    </r>
-  </si>
-  <si>
-    <t>add a pivot table or something foreign in the gSheet sheet</t>
-  </si>
-  <si>
-    <t>&lt;- remember how Tableau failed?  What should I look for in my  application without a schema validation?  I know json is "take what you need and ignore the rest, but what could cause it to catastrophically fail?</t>
-  </si>
-  <si>
-    <t>add data with empty required fields</t>
-  </si>
-  <si>
-    <t>add string in integer field</t>
-  </si>
-  <si>
-    <t>&lt;- There is code for this - gemini showed where but I didn't see it - I should make a console log and test for it.</t>
-  </si>
-  <si>
-    <t>add formula (like an accidental reference) in integer field</t>
-  </si>
-  <si>
-    <t>&lt;- This could happen at source and here as well - both need attention.</t>
-  </si>
-  <si>
-    <t>Fault, not failure - Dia key has Sys value</t>
-  </si>
-  <si>
-    <t>&lt;- Is there any way I can determine if Dia data comes in labeled Sys and vice versa by accident?   They're both 2 digit numbers.</t>
-  </si>
-  <si>
-    <t>&lt;- I check for strings in int fields, but not dates in int fields, do I? I don't have field value requirements written, like int(2) or float(), or string(len) for Comments.</t>
-  </si>
-  <si>
-    <t>Reject future dates.</t>
-  </si>
-  <si>
-    <t>Need validation code - I don't specifically look for it now so these will sneak in currently.</t>
-  </si>
-  <si>
-    <t>Reject dates older than (60?) years</t>
-  </si>
-  <si>
-    <t>Reject "0" value records</t>
-  </si>
-  <si>
-    <t>currently validateNumericReading checks for min: 40 so 0 would be dropped - is that true?  I didn't write a requirement for this!</t>
-  </si>
-  <si>
-    <t>Handle Leap Years</t>
+      <t>Need a log?</t>
+    </r>
   </si>
   <si>
     <r>
@@ -602,7 +734,7 @@
         <rFont val="Calibri"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve">&lt;- Gemini said something about me not rejecting a record if Feb 29 shows up on a non-leap year but instead map() moves it to March 1st.  </t>
+      <t xml:space="preserve">Truncate comments over </t>
     </r>
     <r>
       <rPr>
@@ -611,10 +743,8 @@
         <rFont val="Calibri"/>
         <scheme val="minor"/>
       </rPr>
-      <t>Need a log?</t>
-    </r>
-  </si>
-  <si>
+      <t>How many???</t>
+    </r>
     <r>
       <rPr>
         <sz val="11"/>
@@ -622,24 +752,6 @@
         <rFont val="Calibri"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve">Reject comments over </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>How many???</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
       <t xml:space="preserve"> characters</t>
     </r>
   </si>
@@ -647,75 +759,7 @@
     <t>&lt;- This is huge - this is handling datetime, localization, yyyy-mm-dd, mm/dd/yyyy, etc.  I already cast PM toLower, what else to do???</t>
   </si>
   <si>
-    <t>Application/Functional/Cross Chart Verification</t>
-  </si>
-  <si>
-    <t>Verify Last Reading Date</t>
-  </si>
-  <si>
-    <t>TC-01 x-chart verification</t>
-  </si>
-  <si>
-    <t>ETL from gSheet runs, data.json loaded successfully.</t>
-  </si>
-  <si>
-    <t>Open dashboard, check raw table, check header, check .json</t>
-  </si>
-  <si>
-    <t>Last Reading Date in header matches latest reading date in Raw table, matches latest .json record</t>
-  </si>
-  <si>
-    <t>Header value is "reading date unavailable" on load but has a value after reloading the page.</t>
-  </si>
-  <si>
-    <t>Failed</t>
-  </si>
-  <si>
-    <t>Open a defect.</t>
-  </si>
-  <si>
-    <t>Verify MAX(Date)</t>
-  </si>
-  <si>
-    <t>TC-02 x-chart verification</t>
-  </si>
-  <si>
-    <t>Open dashboard, check raw table, check all x-axis', check .json</t>
-  </si>
-  <si>
-    <t>Raw table, right-most x-axis label, latest Raw table all match latest .json record.</t>
-  </si>
-  <si>
-    <t>Not Run</t>
-  </si>
-  <si>
-    <t>Application/Functional/Date Formatting</t>
-  </si>
-  <si>
-    <t>These are module UI checks because the source has datetime and the x-axis shows different formats, while tooltips show hh-mm-ssAMPM ONLY if it's not an Avg() type chart.</t>
-  </si>
-  <si>
-    <t>TC-01-Datetime Formatting</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Completeness.  </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Calibri"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Or is it called Reconcilliation?</t>
-    </r>
+    <t>Application/Reconcilliation</t>
   </si>
   <si>
     <t>Ensure all records shipped are accounted for; total sent must pass all validation and equal total accepted - happy path.</t>
@@ -738,33 +782,30 @@
     <t>console.log should show the total records received and number rejected, and... the banner should fire a notice "n records rejected for ??? reasons"</t>
   </si>
   <si>
+    <t>There's already a defect but I haven't opened one.  I removed a value from a key, making it null, which dropped it, BUT the total records from the normalizer log didn't decrement and had the whole number of rows back in the source sheet.</t>
+  </si>
+  <si>
+    <t>Application/Security</t>
+  </si>
+  <si>
     <t>Subject</t>
   </si>
   <si>
     <t>Example Subject uses</t>
   </si>
   <si>
-    <t>Design</t>
+    <t>Not Run</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;- IOS+Safari = 1 TC, OSX+Safari=1tc, </t>
   </si>
   <si>
-    <t>Automated</t>
-  </si>
-  <si>
     <t>UI/Functional/Themes</t>
   </si>
   <si>
     <t>&lt;- half implemented.</t>
   </si>
   <si>
-    <t>High</t>
-  </si>
-  <si>
-    <t>UI/Functional/Formatting</t>
-  </si>
-  <si>
     <t>&lt;- data says yyyy-mm-dd, chart.js changes it to mm-dd (tooltips AND x-axis!)</t>
   </si>
   <si>
@@ -777,15 +818,9 @@
     <t>&lt;- async/await loading animation 1 TC + for json arrives before DOM banner "please refresh".  Could lump Cache problems I haven't thought of yet - gemini said something about "Cache Busting" I need to study.</t>
   </si>
   <si>
-    <t>UI/Functional/Reporting</t>
-  </si>
-  <si>
     <t>&lt;- The sum of all Data Integrity the application does (drops, sanitizers).  Is there DQ to show in this?</t>
   </si>
   <si>
-    <t>UI/Functional/Cross Chart verification</t>
-  </si>
-  <si>
     <t>&lt;- this involves inspecting the last record header date, the x-axis and the raw data table - all should agree; had a massive defect with that whole ISO/UTC thing and opened one for Last record date.</t>
   </si>
   <si>
@@ -810,13 +845,7 @@
     <t>&lt;- they trigger, contain correct content, have proper z-index and shader works.</t>
   </si>
   <si>
-    <t>Application/Data Integrity</t>
-  </si>
-  <si>
     <t>&lt;- just logs for each sanitized/validated/dropped/shit, 1 drop = 1 test.  1 sanitize = 1 test, 1 validatin = 1 test..... my NORMALIZATION.  UI/Reporting just rolls it all up.</t>
-  </si>
-  <si>
-    <t>Application/Reconcilliation</t>
   </si>
   <si>
     <t>&lt;- 2 tests - happy path and bad path (accepted + rejected must = total received)</t>
@@ -1530,83 +1559,6 @@
   </si>
   <si>
     <t>Create a pivot table with test counts by folder path</t>
-  </si>
-  <si>
-    <t>errorhandling.js threw this:</t>
-  </si>
-  <si>
-    <t>I don't know what caused it or how to reproduce it.</t>
-  </si>
-  <si>
-    <t>Unhandled Promise Rejection: TypeError: Failed to execute 'fetch' on 'Window': 1 argument required, but only 0 present.</t>
-  </si>
-  <si>
-    <t>I opened a fresh browser tab and went to  http://192.168.2.19:5500/</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    at loadBPData (bp_data_loader.js:31:9)</t>
-  </si>
-  <si>
-    <t>Liveserver is running.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    at bp_data_loader.js:77:3</t>
-  </si>
-  <si>
-    <t>Is this a defect?</t>
-  </si>
-  <si>
-    <t>I was trying to test a 0, sys:null and missing Sys key at the same time by editing the .json file in prod and got this.  It's not my code.</t>
-  </si>
-  <si>
-    <t>I replaced the missing Sys: key and still got it.</t>
-  </si>
-  <si>
-    <t>Here's the thing.... console logged this:</t>
-  </si>
-  <si>
-    <r>
-      <t>bp_data_loader.js:73</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF1F1F1F"/>
-        <rFont val="Courier New"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF410E0B"/>
-        <rFont val="Courier New"/>
-        <charset val="1"/>
-      </rPr>
-      <t>[DATA LOADER] ❌ Failed to load data: SyntaxError: Unexpected token ',', ..." "Sys": , "Dia"... is not valid JSON</t>
-    </r>
-  </si>
-  <si>
-    <t>loadBPData</t>
-  </si>
-  <si>
-    <t>@</t>
-  </si>
-  <si>
-    <t>bp_data_loader.js:73</t>
-  </si>
-  <si>
-    <t>await in loadBPData</t>
-  </si>
-  <si>
-    <t>(anonymous)</t>
-  </si>
-  <si>
-    <t>bp_data_loader.js:76</t>
-  </si>
-  <si>
-    <t>...but the banner didn't fire.  Github's did, but mine didn't!</t>
   </si>
 </sst>
 </file>
@@ -1616,7 +1568,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd;@"/>
   </numFmts>
-  <fonts count="34">
+  <fonts count="29">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1727,13 +1679,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color theme="9"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <b/>
       <sz val="13.5"/>
       <color theme="1"/>
@@ -1800,12 +1745,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color theme="9"/>
-      <name val="Calibri"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <b/>
       <sz val="11"/>
       <color rgb="FFFF0000"/>
@@ -1826,26 +1765,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="9"/>
-      <color rgb="FF1F1F1F"/>
-      <name val="Courier New"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color rgb="FF410E0B"/>
-      <name val="Courier New"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0B57D0"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <b/>
       <sz val="11"/>
       <color rgb="FFFF0000"/>
@@ -1854,7 +1773,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1863,12 +1782,30 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFCEBEB"/>
+        <fgColor theme="0" tint="-4.9989318521683403E-2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -1876,12 +1813,23 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="71">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1953,32 +1901,23 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1987,25 +1926,89 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" quotePrefix="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -2034,25 +2037,222 @@
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>-409575</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>-2857500</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>-409575</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>-2857500</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="2" name="TextBox 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{AEB584D0-A48A-A0F7-13BF-5F9955B9BDB8}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="-409575" y="-2857500"/>
+          <a:ext cx="0" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+        <a:ln w="9525" cmpd="sng">
+          <a:solidFill>
+            <a:schemeClr val="lt1">
+              <a:shade val="50000"/>
+            </a:schemeClr>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:txBody>
+        <a:bodyPr spcFirstLastPara="0" vertOverflow="clip" horzOverflow="clip" wrap="square" lIns="91440" tIns="45720" rIns="91440" bIns="45720" rtlCol="0" anchor="t">
+          <a:noAutofit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr marL="0" indent="0" algn="l"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="0" i="0" u="none" strike="noStrike">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+              <a:ea typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+              <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+            </a:rPr>
+            <a:t>Ok.  I'm sick of scrolling up and down between UI and Application tests.</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr marL="0" indent="0" algn="l"/>
+          <a:endParaRPr lang="en-US" sz="1100" b="0" i="0" u="none" strike="noStrike">
+            <a:solidFill>
+              <a:srgbClr val="000000"/>
+            </a:solidFill>
+            <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+            <a:ea typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+            <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
+          <a:pPr marL="0" indent="0" algn="l"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="0" i="0" u="none" strike="noStrike">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+              <a:ea typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+              <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+            </a:rPr>
+            <a:t>Bring the cooresponding application test up here and put it under the UI one for when one is a UI test and one is a log test.</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr marL="0" indent="0" algn="l"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="0" i="0" u="none" strike="noStrike">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+              <a:ea typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+              <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+            </a:rPr>
+            <a:t>How do I visually tie those together?  I can't merge cells.  It's too soon to assign TC numbers.</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>609600</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>104775</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>2228850</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>514350</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="3" name="TextBox 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4ADF3B2B-C0C3-EC0F-2CB6-AE178D568384}"/>
+            </a:ext>
+            <a:ext uri="{147F2762-F138-4A5C-976F-8EAC2B608ADB}">
+              <a16:predDERef xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" pred="{AEB584D0-A48A-A0F7-13BF-5F9955B9BDB8}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="5000625" y="1857375"/>
+          <a:ext cx="7077075" cy="3905250"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln/>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent2">
+            <a:shade val="15000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent2"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent2"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr spcFirstLastPara="0" vertOverflow="clip" horzOverflow="clip" wrap="square" lIns="91440" tIns="45720" rIns="91440" bIns="45720" rtlCol="0" anchor="t">
+          <a:noAutofit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr marL="0" indent="0" algn="l"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="1600" b="0" i="0" u="none" strike="noStrike">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+              <a:ea typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+              <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+            </a:rPr>
+            <a:t>B</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1600" b="0" i="0" u="none" strike="noStrike">
+              <a:solidFill>
+                <a:schemeClr val="bg1"/>
+              </a:solidFill>
+              <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+              <a:ea typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+              <a:cs typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
+            </a:rPr>
+            <a:t>ring the application tests up underneath the cooresponding UI one because scrolling is causing me to miss shit.</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>104775</xdr:colOff>
-      <xdr:row>6</xdr:row>
-      <xdr:rowOff>28575</xdr:rowOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>723900</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>180975</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>476250</xdr:colOff>
-      <xdr:row>27</xdr:row>
-      <xdr:rowOff>57150</xdr:rowOff>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>1743075</xdr:colOff>
+      <xdr:row>47</xdr:row>
+      <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
         <xdr:cNvPr id="2" name="Picture 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{83D914AF-C792-405F-582E-4E1D0A9F8C2D}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{48E2FFA0-C455-FEB8-695B-91CD2BFC0DD2}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -2068,57 +2268,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="104775" y="1952625"/>
-          <a:ext cx="8905875" cy="4029075"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>4</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>19</xdr:col>
-      <xdr:colOff>438150</xdr:colOff>
-      <xdr:row>24</xdr:row>
-      <xdr:rowOff>114300</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Picture 1">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{036B1418-6078-48E3-2D47-5D8F0F7D9E95}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="962025" y="762000"/>
-          <a:ext cx="11668125" cy="3924300"/>
+          <a:off x="9372600" y="5553075"/>
+          <a:ext cx="4562475" cy="3724275"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2447,10 +2598,7 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <threadedComment ref="E1" dT="2026-03-06T06:05:30.17" personId="{7F340D71-27C9-40D5-A768-16BA27F2EBD1}" id="{0AB13653-40C4-47FA-A319-C6506C77DB43}">
-    <text>gemini suggested keeping the same depth - not only for pivot tables, but it makes your GitHub repo look like it was designed by someone who knows how to architect a test suite, not just list tasks.</text>
-  </threadedComment>
-  <threadedComment ref="F1" dT="2026-03-06T07:29:13.57" personId="{7F340D71-27C9-40D5-A768-16BA27F2EBD1}" id="{B2C5348B-3D7D-45CA-ACA4-7E3CA42663CE}">
+  <threadedComment ref="E1" dT="2026-03-06T07:29:13.57" personId="{7F340D71-27C9-40D5-A768-16BA27F2EBD1}" id="{B2C5348B-3D7D-45CA-ACA4-7E3CA42663CE}">
     <text>A high-level summary of what the test covers.  This is that big blob field in ALM.</text>
   </threadedComment>
 </ThreadedComments>
@@ -2469,29 +2617,29 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:P54"/>
+  <dimension ref="A1:O47"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="2" width="9.140625" style="6"/>
+    <col min="1" max="1" width="9.140625" style="6"/>
+    <col min="2" max="2" width="10.7109375" style="6" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12.140625" style="6" customWidth="1"/>
-    <col min="4" max="4" width="61.42578125" style="6" customWidth="1"/>
-    <col min="5" max="5" width="45.5703125" style="6" customWidth="1"/>
-    <col min="6" max="6" width="45.28515625" style="6" customWidth="1"/>
-    <col min="7" max="7" width="36.5703125" style="6" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="34.140625" style="6" customWidth="1"/>
-    <col min="9" max="9" width="47.7109375" style="6" customWidth="1"/>
-    <col min="10" max="10" width="50.28515625" style="6" customWidth="1"/>
-    <col min="11" max="11" width="45.42578125" style="6" customWidth="1"/>
-    <col min="12" max="12" width="50.28515625" style="6" customWidth="1"/>
-    <col min="13" max="13" width="36.5703125" style="6" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="11.28515625" style="6" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="10.85546875" style="7" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="13.7109375" style="6" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="24.140625" style="6" bestFit="1" customWidth="1"/>
-    <col min="18" max="16384" width="9.140625" style="6"/>
+    <col min="4" max="4" width="33.85546875" style="6" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="45.28515625" style="6" customWidth="1"/>
+    <col min="6" max="6" width="36.5703125" style="6" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="34.140625" style="6" customWidth="1"/>
+    <col min="8" max="8" width="47.7109375" style="6" customWidth="1"/>
+    <col min="9" max="9" width="50.28515625" style="6" customWidth="1"/>
+    <col min="10" max="10" width="45.42578125" style="6" customWidth="1"/>
+    <col min="11" max="11" width="50.28515625" style="6" customWidth="1"/>
+    <col min="12" max="12" width="36.5703125" style="6" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="11.28515625" style="6" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="10.85546875" style="7" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="13.7109375" style="6" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="24.140625" style="6" bestFit="1" customWidth="1"/>
+    <col min="17" max="16384" width="9.140625" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16">
+    <row r="1" spans="1:15">
       <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
@@ -2501,10 +2649,10 @@
       <c r="C1" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="44" t="s">
+      <c r="D1" s="41" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="44" t="s">
+      <c r="E1" s="6" t="s">
         <v>4</v>
       </c>
       <c r="F1" s="6" t="s">
@@ -2531,731 +2679,936 @@
       <c r="M1" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="6" t="s">
+      <c r="N1" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="7" t="s">
+      <c r="O1" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="6" t="s">
+    </row>
+    <row r="2" spans="1:15" s="48" customFormat="1" ht="45.75">
+      <c r="A2" s="48" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="2" spans="1:16" ht="30.75">
-      <c r="A2" s="6" t="s">
+      <c r="B2" s="48" t="s">
         <v>16</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="C2" s="48" t="s">
         <v>17</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="D2" s="48" t="s">
         <v>18</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="E2" s="49" t="s">
         <v>19</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="F2" s="48" t="s">
         <v>20</v>
       </c>
-      <c r="F2" s="8" t="s">
+      <c r="G2" s="53" t="s">
         <v>21</v>
       </c>
-      <c r="G2" s="6" t="s">
+      <c r="I2" s="48" t="s">
         <v>22</v>
       </c>
-      <c r="H2" s="16" t="s">
+      <c r="J2" s="54" t="s">
         <v>23</v>
       </c>
-      <c r="J2" s="6" t="s">
+      <c r="K2" s="55" t="s">
         <v>24</v>
       </c>
-      <c r="K2" s="9" t="s">
+      <c r="M2" s="48" t="s">
         <v>25</v>
       </c>
-      <c r="L2" s="10" t="s">
+      <c r="N2" s="51">
+        <v>46089</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15" ht="45.75">
+      <c r="A3" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="E3" s="49" t="s">
+        <v>19</v>
+      </c>
+      <c r="F3" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="N2" s="6" t="s">
+      <c r="G3" s="16" t="s">
         <v>27</v>
       </c>
-      <c r="O2" s="7">
+      <c r="I3" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="J3" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="K3" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="M3" s="6" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" s="48" customFormat="1" ht="45.75">
+      <c r="A4" s="48" t="s">
+        <v>15</v>
+      </c>
+      <c r="B4" s="48" t="s">
+        <v>16</v>
+      </c>
+      <c r="C4" s="48" t="s">
+        <v>17</v>
+      </c>
+      <c r="D4" s="48" t="s">
+        <v>18</v>
+      </c>
+      <c r="E4" s="49" t="s">
+        <v>19</v>
+      </c>
+      <c r="F4" s="48" t="s">
+        <v>29</v>
+      </c>
+      <c r="G4" s="53" t="s">
+        <v>30</v>
+      </c>
+      <c r="I4" s="48" t="s">
+        <v>22</v>
+      </c>
+      <c r="J4" s="54" t="s">
+        <v>23</v>
+      </c>
+      <c r="K4" s="55" t="s">
+        <v>24</v>
+      </c>
+      <c r="M4" s="48" t="s">
+        <v>25</v>
+      </c>
+      <c r="N4" s="51">
         <v>46089</v>
       </c>
     </row>
-    <row r="3" spans="1:16" ht="30.75">
-      <c r="A3" s="6" t="s">
+    <row r="5" spans="1:15" s="48" customFormat="1" ht="45.75">
+      <c r="A5" s="48" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5" s="48" t="s">
         <v>16</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="C5" s="48" t="s">
         <v>17</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="D5" s="48" t="s">
         <v>18</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="E5" s="49" t="s">
         <v>19</v>
       </c>
-      <c r="E3" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="F3" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="G3" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="H3" s="16" t="s">
-        <v>30</v>
-      </c>
-      <c r="J3" s="6" t="s">
+      <c r="F5" s="48" t="s">
+        <v>31</v>
+      </c>
+      <c r="G5" s="53" t="s">
+        <v>32</v>
+      </c>
+      <c r="I5" s="48" t="s">
+        <v>22</v>
+      </c>
+      <c r="J5" s="54" t="s">
+        <v>23</v>
+      </c>
+      <c r="K5" s="55" t="s">
         <v>24</v>
       </c>
-      <c r="K3" s="9" t="s">
+      <c r="M5" s="48" t="s">
         <v>25</v>
       </c>
-      <c r="L3" s="10" t="s">
+      <c r="N5" s="51">
+        <v>46089</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" s="48" customFormat="1" ht="30.75">
+      <c r="A6" s="48" t="s">
+        <v>33</v>
+      </c>
+      <c r="B6" s="48" t="s">
+        <v>16</v>
+      </c>
+      <c r="C6" s="48" t="s">
+        <v>17</v>
+      </c>
+      <c r="D6" s="48" t="s">
+        <v>18</v>
+      </c>
+      <c r="E6" s="49" t="s">
+        <v>34</v>
+      </c>
+      <c r="F6" s="48" t="s">
+        <v>35</v>
+      </c>
+      <c r="G6" s="53" t="s">
+        <v>36</v>
+      </c>
+      <c r="H6" s="48" t="s">
+        <v>37</v>
+      </c>
+      <c r="J6" s="56" t="s">
+        <v>38</v>
+      </c>
+      <c r="K6" s="66" t="s">
+        <v>39</v>
+      </c>
+      <c r="M6" s="48" t="s">
+        <v>25</v>
+      </c>
+      <c r="N6" s="51">
+        <v>46089</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" s="48" customFormat="1" ht="30.75">
+      <c r="A7" s="48" t="s">
+        <v>40</v>
+      </c>
+      <c r="B7" s="48" t="s">
+        <v>16</v>
+      </c>
+      <c r="C7" s="48" t="s">
+        <v>17</v>
+      </c>
+      <c r="D7" s="48" t="s">
+        <v>41</v>
+      </c>
+      <c r="E7" s="66" t="s">
+        <v>42</v>
+      </c>
+      <c r="H7" s="49" t="s">
+        <v>43</v>
+      </c>
+      <c r="J7" s="49" t="s">
+        <v>44</v>
+      </c>
+      <c r="K7" s="49" t="s">
+        <v>45</v>
+      </c>
+      <c r="L7" s="48" t="s">
+        <v>46</v>
+      </c>
+      <c r="M7" s="48" t="s">
+        <v>25</v>
+      </c>
+      <c r="N7" s="51">
+        <v>46089</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15" ht="60.75">
+      <c r="C8" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="E8" s="26" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15">
+      <c r="C9" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="D9" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="E9" s="26" t="s">
+        <v>50</v>
+      </c>
+      <c r="H9" s="8"/>
+    </row>
+    <row r="10" spans="1:15" s="45" customFormat="1" ht="76.5">
+      <c r="A10" s="45" t="s">
+        <v>40</v>
+      </c>
+      <c r="B10" s="45" t="s">
+        <v>16</v>
+      </c>
+      <c r="C10" s="45" t="s">
+        <v>17</v>
+      </c>
+      <c r="D10" s="45" t="s">
+        <v>51</v>
+      </c>
+      <c r="E10" s="46" t="s">
+        <v>52</v>
+      </c>
+      <c r="G10" s="46" t="s">
+        <v>53</v>
+      </c>
+      <c r="H10" s="62" t="s">
+        <v>54</v>
+      </c>
+      <c r="J10" s="46" t="s">
+        <v>55</v>
+      </c>
+      <c r="K10" s="67" t="s">
+        <v>56</v>
+      </c>
+      <c r="L10" s="46" t="s">
+        <v>57</v>
+      </c>
+      <c r="M10" s="45" t="s">
+        <v>25</v>
+      </c>
+      <c r="N10" s="47">
+        <v>46089</v>
+      </c>
+      <c r="O10" s="45">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15" s="48" customFormat="1" ht="30.75">
+      <c r="A11" s="48" t="s">
+        <v>40</v>
+      </c>
+      <c r="B11" s="48" t="s">
+        <v>16</v>
+      </c>
+      <c r="C11" s="48" t="s">
+        <v>17</v>
+      </c>
+      <c r="D11" s="48" t="s">
+        <v>51</v>
+      </c>
+      <c r="E11" s="49" t="s">
+        <v>58</v>
+      </c>
+      <c r="G11" s="49" t="s">
+        <v>59</v>
+      </c>
+      <c r="H11" s="48" t="s">
+        <v>60</v>
+      </c>
+      <c r="J11" s="49" t="s">
+        <v>61</v>
+      </c>
+      <c r="K11" s="52" t="s">
+        <v>62</v>
+      </c>
+      <c r="L11" s="49" t="s">
+        <v>57</v>
+      </c>
+      <c r="M11" s="48" t="s">
+        <v>25</v>
+      </c>
+      <c r="N11" s="51">
+        <v>46093</v>
+      </c>
+      <c r="O11" s="48">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15" s="45" customFormat="1" ht="30.75">
+      <c r="A12" s="45" t="s">
+        <v>40</v>
+      </c>
+      <c r="B12" s="45" t="s">
+        <v>16</v>
+      </c>
+      <c r="C12" s="45" t="s">
+        <v>17</v>
+      </c>
+      <c r="D12" s="45" t="s">
+        <v>51</v>
+      </c>
+      <c r="E12" s="46" t="s">
+        <v>63</v>
+      </c>
+      <c r="G12" s="46" t="s">
+        <v>64</v>
+      </c>
+      <c r="H12" s="67" t="s">
+        <v>65</v>
+      </c>
+      <c r="J12" s="46" t="s">
+        <v>66</v>
+      </c>
+      <c r="K12" s="67" t="s">
+        <v>67</v>
+      </c>
+      <c r="L12" s="46" t="s">
+        <v>57</v>
+      </c>
+      <c r="M12" s="45" t="s">
+        <v>25</v>
+      </c>
+      <c r="N12" s="47">
+        <v>46093</v>
+      </c>
+      <c r="O12" s="45">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15" ht="45.75">
+      <c r="C13" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="D13" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="E13" s="68" t="s">
+        <v>68</v>
+      </c>
+      <c r="I13" s="8"/>
+      <c r="J13" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="K13" s="26" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="14" spans="1:15" ht="152.25">
+      <c r="C14" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="D14" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="E14" s="36" t="s">
+        <v>72</v>
+      </c>
+      <c r="H14" s="8"/>
+    </row>
+    <row r="15" spans="1:15" s="57" customFormat="1" ht="45.75">
+      <c r="A15" s="57" t="s">
+        <v>33</v>
+      </c>
+      <c r="B15" s="57" t="s">
+        <v>16</v>
+      </c>
+      <c r="C15" s="57" t="s">
+        <v>17</v>
+      </c>
+      <c r="D15" s="57" t="s">
+        <v>73</v>
+      </c>
+      <c r="E15" s="57" t="s">
+        <v>74</v>
+      </c>
+      <c r="F15" s="57" t="s">
+        <v>20</v>
+      </c>
+      <c r="G15" s="58" t="s">
+        <v>75</v>
+      </c>
+      <c r="I15" s="58" t="s">
+        <v>76</v>
+      </c>
+      <c r="J15" s="58" t="s">
+        <v>77</v>
+      </c>
+      <c r="K15" s="58" t="s">
+        <v>78</v>
+      </c>
+      <c r="L15" s="58" t="s">
+        <v>79</v>
+      </c>
+      <c r="M15" s="57" t="s">
+        <v>80</v>
+      </c>
+      <c r="N15" s="59">
+        <v>46093</v>
+      </c>
+      <c r="O15" s="60" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="16" spans="1:15" ht="60.75">
+      <c r="A16" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="B16" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="C16" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="D16" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="E16" s="68" t="s">
+        <v>82</v>
+      </c>
+      <c r="F16" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="N3" s="6" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="4" spans="1:16" ht="30.75">
-      <c r="A4" s="6" t="s">
+      <c r="G16" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="I16" s="8" t="s">
+        <v>76</v>
+      </c>
+      <c r="J16" s="8"/>
+      <c r="K16" s="8"/>
+    </row>
+    <row r="17" spans="1:14" ht="60.75">
+      <c r="C17" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="D17" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="E17" s="26" t="s">
+        <v>85</v>
+      </c>
+      <c r="F17" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="G17" s="8" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="18" spans="1:14" s="42" customFormat="1">
+      <c r="E18" s="43"/>
+      <c r="N18" s="44"/>
+    </row>
+    <row r="19" spans="1:14" ht="106.5">
+      <c r="C19" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="D19" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="E19" s="36" t="s">
+        <v>88</v>
+      </c>
+      <c r="J19" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="K19" s="68"/>
+    </row>
+    <row r="20" spans="1:14" ht="60.75">
+      <c r="C20" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="D20" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="E20" s="8" t="s">
+        <v>90</v>
+      </c>
+      <c r="H20" s="8" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="21" spans="1:14" ht="137.25">
+      <c r="C21" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="D21" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="E21" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="H21" s="26" t="s">
+        <v>93</v>
+      </c>
+      <c r="K21" s="68" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="22" spans="1:14">
+      <c r="C22" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="D22" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="E22" s="11" t="s">
+        <v>96</v>
+      </c>
+      <c r="I22" s="8"/>
+      <c r="J22" s="8"/>
+      <c r="K22" s="8"/>
+    </row>
+    <row r="23" spans="1:14" ht="45.75">
+      <c r="C23" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="D23" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="E23" s="26" t="s">
+        <v>97</v>
+      </c>
+      <c r="H23" s="11"/>
+      <c r="I23" s="8"/>
+      <c r="J23" s="8"/>
+      <c r="K23" s="8"/>
+    </row>
+    <row r="24" spans="1:14" s="57" customFormat="1" ht="76.5">
+      <c r="A24" s="57" t="s">
+        <v>40</v>
+      </c>
+      <c r="B24" s="57" t="s">
         <v>16</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="C24" s="57" t="s">
         <v>17</v>
       </c>
-      <c r="C4" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="D4" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="E4" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="F4" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="G4" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="H4" s="16" t="s">
-        <v>34</v>
-      </c>
-      <c r="J4" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="K4" s="9" t="s">
+      <c r="D24" s="57" t="s">
+        <v>95</v>
+      </c>
+      <c r="E24" s="58" t="s">
+        <v>98</v>
+      </c>
+      <c r="G24" s="58" t="s">
+        <v>53</v>
+      </c>
+      <c r="H24" s="64" t="s">
+        <v>54</v>
+      </c>
+      <c r="J24" s="58" t="s">
+        <v>99</v>
+      </c>
+      <c r="K24" s="60" t="s">
+        <v>100</v>
+      </c>
+      <c r="L24" s="58"/>
+      <c r="N24" s="59">
+        <v>46089</v>
+      </c>
+    </row>
+    <row r="25" spans="1:14" s="50" customFormat="1" ht="32.25">
+      <c r="A25" s="50" t="s">
+        <v>40</v>
+      </c>
+      <c r="B25" s="50" t="s">
+        <v>16</v>
+      </c>
+      <c r="C25" s="50" t="s">
+        <v>47</v>
+      </c>
+      <c r="D25" s="50" t="s">
+        <v>95</v>
+      </c>
+      <c r="E25" s="52" t="s">
+        <v>58</v>
+      </c>
+      <c r="G25" s="52" t="s">
+        <v>59</v>
+      </c>
+      <c r="H25" s="50" t="s">
+        <v>60</v>
+      </c>
+      <c r="J25" s="52" t="s">
+        <v>101</v>
+      </c>
+      <c r="K25" s="52" t="s">
+        <v>102</v>
+      </c>
+      <c r="L25" s="50" t="s">
+        <v>103</v>
+      </c>
+      <c r="M25" s="50" t="s">
         <v>25</v>
       </c>
-      <c r="L4" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="N4" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="O4" s="7">
+      <c r="N25" s="63">
         <v>46089</v>
       </c>
     </row>
-    <row r="5" spans="1:16" ht="30.75">
-      <c r="A5" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="B5" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="C5" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="D5" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="E5" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="F5" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="G5" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="H5" s="16" t="s">
-        <v>37</v>
-      </c>
-      <c r="J5" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="K5" s="9" t="s">
-        <v>25</v>
-      </c>
-      <c r="L5" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="N5" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="O5" s="7">
-        <v>46089</v>
-      </c>
-    </row>
-    <row r="6" spans="1:16" ht="30.75">
-      <c r="A6" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="B6" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="C6" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="D6" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="F6" s="8" t="s">
-        <v>39</v>
-      </c>
-      <c r="G6" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="H6" s="16" t="s">
-        <v>41</v>
-      </c>
-      <c r="I6" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="K6" s="45" t="s">
-        <v>43</v>
-      </c>
-      <c r="L6" s="52" t="s">
-        <v>44</v>
-      </c>
-      <c r="N6" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="O6" s="7">
-        <v>46089</v>
-      </c>
-    </row>
-    <row r="7" spans="1:16" ht="30.75">
-      <c r="A7" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="B7" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="C7" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="D7" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="E7" s="6" t="s">
-        <v>46</v>
-      </c>
-      <c r="F7" s="52" t="s">
+    <row r="26" spans="1:14" s="45" customFormat="1" ht="45.75">
+      <c r="A26" s="45" t="s">
+        <v>15</v>
+      </c>
+      <c r="B26" s="45" t="s">
+        <v>104</v>
+      </c>
+      <c r="C26" s="45" t="s">
         <v>47</v>
       </c>
-      <c r="I7" s="8" t="s">
-        <v>48</v>
-      </c>
-      <c r="K7" s="8" t="s">
-        <v>49</v>
-      </c>
-      <c r="L7" s="8" t="s">
-        <v>50</v>
-      </c>
-      <c r="M7" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="N7" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="O7" s="7">
-        <v>46089</v>
-      </c>
-    </row>
-    <row r="8" spans="1:16" ht="60.75">
-      <c r="D8" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="E8" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="F8" s="26" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="9" spans="1:16">
-      <c r="D9" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="F9" s="26" t="s">
-        <v>55</v>
-      </c>
-      <c r="I9" s="8"/>
-    </row>
-    <row r="10" spans="1:16" ht="60.75">
-      <c r="D10" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="F10" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="H10" s="8" t="s">
-        <v>58</v>
-      </c>
-      <c r="I10" s="8"/>
-      <c r="K10" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="L10" s="6" t="s">
-        <v>60</v>
-      </c>
-      <c r="M10" s="8" t="s">
-        <v>61</v>
-      </c>
-      <c r="N10" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="O10" s="7">
-        <v>46089</v>
-      </c>
-      <c r="P10" s="6">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="11" spans="1:16">
-      <c r="F11" s="8"/>
-      <c r="I11" s="8"/>
-    </row>
-    <row r="12" spans="1:16">
-      <c r="F12" s="8"/>
-      <c r="I12" s="8"/>
-    </row>
-    <row r="13" spans="1:16" ht="106.5">
-      <c r="D13" s="6" t="s">
-        <v>62</v>
-      </c>
-      <c r="E13" s="27" t="s">
-        <v>62</v>
-      </c>
-      <c r="F13" s="46" t="s">
+      <c r="D26" s="45" t="s">
+        <v>95</v>
+      </c>
+      <c r="E26" s="46" t="s">
         <v>63</v>
       </c>
-      <c r="G13" s="6" t="s">
+      <c r="G26" s="46" t="s">
         <v>64</v>
       </c>
-      <c r="K13" s="6" t="s">
-        <v>65</v>
-      </c>
-      <c r="L13" s="52"/>
-    </row>
-    <row r="14" spans="1:16" ht="60.75">
-      <c r="D14" s="6" t="s">
-        <v>62</v>
-      </c>
-      <c r="E14" s="27" t="s">
-        <v>66</v>
-      </c>
-      <c r="F14" s="8" t="s">
-        <v>67</v>
-      </c>
-      <c r="I14" s="8" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="15" spans="1:16" ht="137.25">
-      <c r="D15" s="6" t="s">
-        <v>62</v>
-      </c>
-      <c r="E15" s="27" t="s">
-        <v>62</v>
-      </c>
-      <c r="F15" s="8" t="s">
-        <v>69</v>
-      </c>
-      <c r="I15" s="8" t="s">
-        <v>70</v>
-      </c>
-      <c r="L15" s="52" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="16" spans="1:16" ht="45.75">
-      <c r="D16" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="E16" s="27" t="s">
-        <v>72</v>
-      </c>
-      <c r="F16" s="52" t="s">
-        <v>73</v>
-      </c>
-      <c r="J16" s="8"/>
-      <c r="K16" s="8" t="s">
-        <v>74</v>
-      </c>
-      <c r="L16" s="8" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="17" spans="4:15">
-      <c r="E17" s="27" t="s">
-        <v>76</v>
-      </c>
-      <c r="I17" s="11" t="s">
-        <v>77</v>
-      </c>
-      <c r="J17" s="8"/>
-      <c r="K17" s="8"/>
-      <c r="L17" s="8"/>
-    </row>
-    <row r="18" spans="4:15" ht="45.75">
-      <c r="D18" s="6" t="s">
-        <v>78</v>
-      </c>
-      <c r="E18" s="27"/>
-      <c r="F18" s="26" t="s">
-        <v>79</v>
-      </c>
-      <c r="I18" s="11"/>
-      <c r="J18" s="8"/>
-      <c r="K18" s="8"/>
-      <c r="L18" s="8"/>
-    </row>
-    <row r="19" spans="4:15" ht="60.75">
-      <c r="D19" s="6" t="s">
-        <v>78</v>
-      </c>
-      <c r="E19" s="27"/>
-      <c r="F19" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="H19" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="I19" s="11"/>
-      <c r="J19"/>
-      <c r="K19" s="8" t="s">
-        <v>82</v>
-      </c>
-      <c r="L19" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="M19" s="8" t="s">
-        <v>84</v>
-      </c>
-      <c r="N19" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="O19" s="7">
-        <v>46089</v>
-      </c>
-    </row>
-    <row r="20" spans="4:15" ht="45.75">
-      <c r="E20" s="27" t="s">
-        <v>85</v>
-      </c>
-      <c r="I20" s="6" t="s">
-        <v>86</v>
-      </c>
-      <c r="K20" s="8" t="s">
-        <v>87</v>
-      </c>
-      <c r="L20" s="8" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="21" spans="4:15" ht="137.25">
-      <c r="E21" s="27" t="s">
-        <v>85</v>
-      </c>
-      <c r="I21" s="6" t="s">
-        <v>89</v>
-      </c>
-      <c r="K21" s="8" t="s">
-        <v>87</v>
-      </c>
-      <c r="L21" s="39" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="22" spans="4:15" ht="121.5">
-      <c r="E22" s="36" t="s">
-        <v>91</v>
-      </c>
-      <c r="F22" s="8"/>
-      <c r="I22" s="37" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="23" spans="4:15" ht="60.75">
-      <c r="E23" s="36" t="s">
-        <v>91</v>
-      </c>
-      <c r="F23" s="8" t="s">
-        <v>93</v>
-      </c>
-      <c r="I23" s="8" t="s">
-        <v>94</v>
-      </c>
-      <c r="L23" s="8"/>
-    </row>
-    <row r="24" spans="4:15">
-      <c r="E24" s="36" t="s">
-        <v>91</v>
-      </c>
-      <c r="F24" s="6" t="s">
-        <v>95</v>
-      </c>
-      <c r="L24" s="8"/>
-    </row>
-    <row r="25" spans="4:15" ht="45.75">
-      <c r="E25" s="36" t="s">
-        <v>91</v>
-      </c>
-      <c r="F25" s="6" t="s">
-        <v>96</v>
-      </c>
-      <c r="I25" s="8" t="s">
-        <v>97</v>
-      </c>
-      <c r="L25" s="8"/>
-    </row>
-    <row r="26" spans="4:15" ht="30.75">
-      <c r="E26" s="36" t="s">
-        <v>91</v>
-      </c>
-      <c r="F26" s="8" t="s">
-        <v>98</v>
-      </c>
-      <c r="I26" s="8" t="s">
-        <v>99</v>
-      </c>
-      <c r="L26" s="8"/>
-    </row>
-    <row r="27" spans="4:15" s="8" customFormat="1" ht="45.75">
-      <c r="D27" s="6"/>
-      <c r="E27" s="36" t="s">
-        <v>91</v>
-      </c>
-      <c r="F27" s="8" t="s">
-        <v>100</v>
-      </c>
-      <c r="I27" s="8" t="s">
-        <v>101</v>
-      </c>
-      <c r="O27" s="22"/>
-    </row>
-    <row r="28" spans="4:15" s="8" customFormat="1" ht="60.75">
-      <c r="D28" s="6"/>
-      <c r="E28" s="36" t="s">
-        <v>91</v>
-      </c>
-      <c r="F28" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="I28" s="8" t="s">
-        <v>102</v>
-      </c>
-      <c r="O28" s="22"/>
-    </row>
-    <row r="29" spans="4:15" ht="30.75">
-      <c r="E29" s="36" t="s">
-        <v>91</v>
-      </c>
-      <c r="F29" s="6" t="s">
-        <v>103</v>
-      </c>
-      <c r="I29" s="26" t="s">
-        <v>104</v>
-      </c>
-      <c r="J29" s="8"/>
-    </row>
-    <row r="30" spans="4:15" ht="30.75">
-      <c r="E30" s="36" t="s">
-        <v>91</v>
-      </c>
-      <c r="F30" s="6" t="s">
+      <c r="H26" s="45" t="s">
         <v>105</v>
       </c>
-      <c r="I30" s="26" t="s">
-        <v>104</v>
-      </c>
-      <c r="J30" s="8"/>
-    </row>
-    <row r="31" spans="4:15" ht="45.75">
-      <c r="E31" s="36" t="s">
-        <v>91</v>
-      </c>
-      <c r="F31" s="6" t="s">
+      <c r="J26" s="46" t="s">
         <v>106</v>
       </c>
-      <c r="I31" s="26" t="s">
+      <c r="K26" s="61" t="s">
         <v>107</v>
       </c>
-      <c r="J31" s="8"/>
-    </row>
-    <row r="32" spans="4:15" ht="45.75">
-      <c r="E32" s="36" t="s">
-        <v>91</v>
-      </c>
-      <c r="F32" s="6" t="s">
+      <c r="N26" s="47"/>
+    </row>
+    <row r="27" spans="1:14" ht="121.5">
+      <c r="C27" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="D27" s="6" t="s">
         <v>108</v>
       </c>
-      <c r="I32" s="52" t="s">
+      <c r="E27" s="8"/>
+      <c r="H27" s="35" t="s">
         <v>109</v>
       </c>
-      <c r="J32" s="8"/>
-    </row>
-    <row r="33" spans="3:16">
-      <c r="E33" s="36" t="s">
-        <v>91</v>
-      </c>
-      <c r="F33" s="47" t="s">
+    </row>
+    <row r="28" spans="1:14" ht="60.75">
+      <c r="C28" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="D28" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="E28" s="8" t="s">
         <v>110</v>
       </c>
-      <c r="I33" s="52"/>
-      <c r="J33" s="8"/>
-    </row>
-    <row r="34" spans="3:16" ht="45.75">
-      <c r="E34" s="36" t="s">
-        <v>91</v>
-      </c>
-      <c r="F34" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="I34" s="8" t="s">
+      <c r="H28" s="8" t="s">
         <v>111</v>
       </c>
-    </row>
-    <row r="35" spans="3:16" ht="45.75">
-      <c r="E35" s="38" t="s">
+      <c r="K28" s="8"/>
+    </row>
+    <row r="29" spans="1:14">
+      <c r="C29" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="D29" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="E29" s="6" t="s">
         <v>112</v>
       </c>
-      <c r="F35" s="6" t="s">
+      <c r="K29" s="8"/>
+    </row>
+    <row r="30" spans="1:14" ht="45.75">
+      <c r="C30" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="D30" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="E30" s="6" t="s">
         <v>113</v>
       </c>
-      <c r="G35" s="6" t="s">
+      <c r="H30" s="8" t="s">
         <v>114</v>
       </c>
-      <c r="J35" s="8" t="s">
+      <c r="K30" s="8"/>
+    </row>
+    <row r="31" spans="1:14" ht="30.75">
+      <c r="C31" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="D31" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="E31" s="8" t="s">
         <v>115</v>
       </c>
-      <c r="K35" s="8" t="s">
+      <c r="H31" s="8" t="s">
         <v>116</v>
       </c>
-      <c r="L35" s="8" t="s">
+      <c r="K31" s="8"/>
+    </row>
+    <row r="32" spans="1:14" s="8" customFormat="1" ht="45.75">
+      <c r="B32" s="6"/>
+      <c r="C32" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="D32" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="E32" s="8" t="s">
         <v>117</v>
       </c>
-      <c r="M35" s="8" t="s">
+      <c r="H32" s="8" t="s">
         <v>118</v>
       </c>
-      <c r="N35" s="6" t="s">
+      <c r="N32" s="22"/>
+    </row>
+    <row r="33" spans="2:14" s="8" customFormat="1" ht="60.75">
+      <c r="B33" s="6"/>
+      <c r="C33" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="D33" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="E33" s="8" t="s">
         <v>119</v>
       </c>
-      <c r="P35" s="26" t="s">
+      <c r="H33" s="8" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="36" spans="3:16" ht="30.75">
-      <c r="E36" s="38" t="s">
-        <v>112</v>
-      </c>
-      <c r="F36" s="6" t="s">
+      <c r="N33" s="22"/>
+    </row>
+    <row r="34" spans="2:14" ht="30.75">
+      <c r="C34" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="D34" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="E34" s="6" t="s">
         <v>121</v>
       </c>
-      <c r="G36" s="6" t="s">
+      <c r="H34" s="26" t="s">
         <v>122</v>
       </c>
-      <c r="J36" s="8" t="s">
-        <v>115</v>
-      </c>
-      <c r="K36" s="8" t="s">
+      <c r="I34" s="8"/>
+    </row>
+    <row r="35" spans="2:14" ht="30.75">
+      <c r="C35" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="D35" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="E35" s="6" t="s">
         <v>123</v>
       </c>
-      <c r="L36" s="8" t="s">
+      <c r="H35" s="26" t="s">
+        <v>122</v>
+      </c>
+      <c r="I35" s="8"/>
+    </row>
+    <row r="36" spans="2:14" ht="45.75">
+      <c r="C36" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="D36" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="E36" s="6" t="s">
         <v>124</v>
       </c>
-      <c r="N36" s="6" t="s">
+      <c r="H36" s="26" t="s">
         <v>125</v>
       </c>
-    </row>
-    <row r="37" spans="3:16" ht="60.75">
-      <c r="E37" s="38" t="s">
+      <c r="I36" s="8"/>
+    </row>
+    <row r="37" spans="2:14" ht="45.75">
+      <c r="C37" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="D37" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="E37" s="6" t="s">
         <v>126</v>
       </c>
-      <c r="F37" s="8" t="s">
+      <c r="H37" s="68" t="s">
         <v>127</v>
       </c>
-      <c r="G37" s="6" t="s">
+      <c r="I37" s="8"/>
+    </row>
+    <row r="38" spans="2:14">
+      <c r="C38" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="D38" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="E38" s="69" t="s">
         <v>128</v>
       </c>
-      <c r="N37" s="6" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="38" spans="3:16">
-      <c r="E38" s="36"/>
+      <c r="H38" s="68"/>
       <c r="I38" s="8"/>
     </row>
-    <row r="39" spans="3:16" ht="45.75">
-      <c r="E39" s="52" t="s">
+    <row r="39" spans="2:14" ht="45.75">
+      <c r="C39" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="D39" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="E39" s="6" t="s">
+        <v>119</v>
+      </c>
+      <c r="H39" s="8" t="s">
         <v>129</v>
       </c>
-      <c r="F39" s="8" t="s">
+    </row>
+    <row r="40" spans="2:14" ht="45.75">
+      <c r="C40" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="D40" s="6" t="s">
         <v>130</v>
       </c>
-      <c r="G39" s="8"/>
-      <c r="I39" s="25" t="s">
+      <c r="E40" s="26" t="s">
         <v>131</v>
       </c>
-      <c r="L39" s="6" t="s">
+      <c r="F40" s="8"/>
+      <c r="H40" s="25" t="s">
         <v>132</v>
       </c>
-    </row>
-    <row r="40" spans="3:16" ht="76.5">
-      <c r="E40" s="52" t="s">
-        <v>129</v>
-      </c>
-      <c r="F40" s="8" t="s">
+      <c r="K40" s="6" t="s">
         <v>133</v>
       </c>
-      <c r="I40" s="25" t="s">
-        <v>131</v>
-      </c>
-      <c r="K40" s="53" t="s">
+    </row>
+    <row r="41" spans="2:14" ht="106.5">
+      <c r="C41" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="D41" s="6" t="s">
+        <v>130</v>
+      </c>
+      <c r="E41" s="26" t="s">
         <v>134</v>
       </c>
-      <c r="L40" s="8" t="s">
+      <c r="H41" s="25" t="s">
+        <v>132</v>
+      </c>
+      <c r="J41" s="70" t="s">
         <v>135</v>
       </c>
-    </row>
-    <row r="43" spans="3:16">
-      <c r="C43" s="12"/>
-    </row>
-    <row r="45" spans="3:16">
-      <c r="H45" s="8"/>
-      <c r="L45" s="8"/>
-    </row>
-    <row r="46" spans="3:16">
-      <c r="H46" s="8"/>
-      <c r="L46" s="8"/>
-    </row>
-    <row r="54" spans="6:6">
-      <c r="F54" s="3"/>
+      <c r="K41" s="8" t="s">
+        <v>136</v>
+      </c>
+      <c r="L41" s="65" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="42" spans="2:14">
+      <c r="C42" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="D42" s="6" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="44" spans="2:14">
+      <c r="C44" s="12"/>
+    </row>
+    <row r="46" spans="2:14">
+      <c r="G46" s="8"/>
+      <c r="K46" s="8"/>
+    </row>
+    <row r="47" spans="2:14">
+      <c r="G47" s="8"/>
+      <c r="K47" s="8"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P2" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:O2" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <dataValidations count="1">
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F35:F36 I14 G13 H13:H21 H23:H26 J20:J1048576 F20:H23 P35:P37 K35:M36 E7:E8 E65:E1048576 E12:E38 E45:E60 D1 D54:D1048576 E1:E5 P2:P23 F2:G6 K2:M6 J1:J18 K13:K23 K10 L13:L18 L20:L23 H10 M13:M23 N22:N23" xr:uid="{F7B3DB26-BE56-424E-8D9E-1D07DC9827CF}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H20 F19 K11 D1 D55:D1048576 K26:K28 J2:L6 I1:I12 J10:J13 M27:M28 B27:B41 K22:K23 I13:L13 J19:L21 J22:J28 G19:G31 G10:G13 E27:E28 F25:F28 B17:B23 I14:I23 L22:L28 E15:E16 J15:L16 I25:I1048576 O2:O28 B13:B14 B8:B9 E2:F6" xr:uid="{F7B3DB26-BE56-424E-8D9E-1D07DC9827CF}"/>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <legacyDrawing r:id="rId1"/>
+  <drawing r:id="rId1"/>
+  <legacyDrawing r:id="rId2"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="5">
@@ -3263,31 +3616,31 @@
           <x14:formula1>
             <xm:f>ValidationDDLsource!$E$2:$E$18</xm:f>
           </x14:formula1>
-          <xm:sqref>N35:N37 N2:N23</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{EA1E7D53-A2D7-43C3-8991-B56E45D2485E}">
-          <x14:formula1>
-            <xm:f>ValidationDDLsource!$A$2:$A$4</xm:f>
-          </x14:formula1>
-          <xm:sqref>C35:C37 C2:C23</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{927E9024-62E5-4B45-92A3-AEDB6A1233F6}">
-          <x14:formula1>
-            <xm:f>ValidationDDLsource!$B$2:$B$3</xm:f>
-          </x14:formula1>
-          <xm:sqref>B35:C37 B2:C23</xm:sqref>
+          <xm:sqref>M2:M28</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{3C46C409-7480-4F5F-B77B-8830A973D994}">
           <x14:formula1>
             <xm:f>ValidationDDLsource!$C$2:$C$5</xm:f>
           </x14:formula1>
-          <xm:sqref>A35:C37 A2:C23</xm:sqref>
+          <xm:sqref>A2:A28</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{84E4F64A-3933-429A-B308-69991B99FB29}">
+          <x14:formula1>
+            <xm:f>ValidationDDLsource!$B$2:$B$7</xm:f>
+          </x14:formula1>
+          <xm:sqref>B2:B7 B15:B16 B10:B12 B24:B26</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{5ABE4842-C5A7-4314-B8E4-942306CCE80B}">
           <x14:formula1>
             <xm:f>ValidationDDLsource!$D$2:$D$39</xm:f>
           </x14:formula1>
-          <xm:sqref>D2:D53</xm:sqref>
+          <xm:sqref>D2:D54</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{2EC0DFA8-4C18-4C59-80D7-71402ADEAE7C}">
+          <x14:formula1>
+            <xm:f>ValidationDDLsource!$A$2:$A$7</xm:f>
+          </x14:formula1>
+          <xm:sqref>C2:C42</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -3320,64 +3673,64 @@
         <v>0</v>
       </c>
       <c r="D1" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="E1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" t="s">
-        <v>138</v>
+        <v>47</v>
       </c>
       <c r="B2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C2" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E2" t="s">
-        <v>125</v>
+        <v>141</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
     </row>
     <row r="3" spans="1:7">
       <c r="A3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B3" t="s">
-        <v>140</v>
+        <v>104</v>
       </c>
       <c r="C3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="E3" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="G3" s="6" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
     </row>
     <row r="4" spans="1:7">
       <c r="C4" t="s">
-        <v>143</v>
+        <v>33</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>144</v>
+        <v>84</v>
       </c>
       <c r="E4" t="s">
-        <v>119</v>
+        <v>80</v>
       </c>
       <c r="G4" s="6" t="s">
         <v>145</v>
@@ -3388,10 +3741,10 @@
         <v>146</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="E5" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="G5" s="6" t="s">
         <v>147</v>
@@ -3399,7 +3752,7 @@
     </row>
     <row r="6" spans="1:7">
       <c r="D6" s="6" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="G6" s="6" t="s">
         <v>148</v>
@@ -3407,99 +3760,101 @@
     </row>
     <row r="7" spans="1:7">
       <c r="D7" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="G7" s="6" t="s">
         <v>149</v>
-      </c>
-      <c r="G7" s="6" t="s">
-        <v>150</v>
       </c>
     </row>
     <row r="8" spans="1:7">
       <c r="D8" s="6" t="s">
-        <v>151</v>
+        <v>73</v>
       </c>
       <c r="G8" s="6" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
     </row>
     <row r="9" spans="1:7">
       <c r="D9" s="6" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="G9" s="6" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
     </row>
     <row r="10" spans="1:7">
       <c r="D10" s="6" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="G10" s="6" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
     </row>
     <row r="11" spans="1:7">
       <c r="D11" s="6" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
     </row>
     <row r="12" spans="1:7">
       <c r="D12" s="6" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
     </row>
     <row r="13" spans="1:7">
       <c r="D13" s="6" t="s">
-        <v>62</v>
+        <v>87</v>
       </c>
     </row>
     <row r="14" spans="1:7">
       <c r="D14" s="6" t="s">
-        <v>78</v>
+        <v>95</v>
       </c>
       <c r="G14" s="6" t="s">
-        <v>77</v>
+        <v>96</v>
       </c>
     </row>
     <row r="15" spans="1:7">
       <c r="D15" s="6" t="s">
-        <v>160</v>
+        <v>108</v>
       </c>
       <c r="G15" s="6" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
     </row>
     <row r="16" spans="1:7">
       <c r="D16" s="6" t="s">
-        <v>162</v>
+        <v>130</v>
       </c>
       <c r="G16" s="6" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
     </row>
     <row r="17" spans="4:7">
       <c r="D17" s="6" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
       <c r="G17" s="6" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
     </row>
     <row r="18" spans="4:7">
-      <c r="D18" s="6"/>
+      <c r="D18" s="6" t="s">
+        <v>138</v>
+      </c>
     </row>
     <row r="19" spans="4:7" ht="21">
       <c r="D19" s="6"/>
-      <c r="G19" s="35"/>
+      <c r="G19" s="34"/>
     </row>
     <row r="20" spans="4:7" ht="18.75">
       <c r="D20" s="6"/>
-      <c r="G20" s="40"/>
+      <c r="G20" s="37"/>
     </row>
     <row r="21" spans="4:7">
       <c r="D21" s="6"/>
@@ -3606,87 +3961,87 @@
         <v>2</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="E1" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="F1" s="6" t="s">
+      <c r="G1" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="G1" s="6" t="s">
+      <c r="H1" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="H1" s="6" t="s">
+      <c r="I1" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="I1" s="6" t="s">
+      <c r="J1" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="J1" s="6" t="s">
+      <c r="K1" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="K1" s="6" t="s">
+      <c r="L1" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="L1" s="6" t="s">
+      <c r="M1" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="M1" s="6" t="s">
+      <c r="N1" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="N1" s="7" t="s">
+      <c r="O1" s="6" t="s">
         <v>14</v>
-      </c>
-      <c r="O1" s="6" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="2" spans="1:15" ht="21">
       <c r="D2" s="17" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
     </row>
     <row r="3" spans="1:15">
       <c r="D3" s="11" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
     </row>
     <row r="4" spans="1:15">
       <c r="D4" s="11" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
     </row>
     <row r="6" spans="1:15" s="18" customFormat="1">
       <c r="D6" s="18" t="s">
+        <v>166</v>
+      </c>
+      <c r="E6" s="18" t="s">
+        <v>167</v>
+      </c>
+      <c r="F6" s="18" t="s">
+        <v>168</v>
+      </c>
+      <c r="G6" s="18" t="s">
+        <v>169</v>
+      </c>
+      <c r="H6" s="18" t="s">
         <v>170</v>
       </c>
-      <c r="E6" s="18" t="s">
+      <c r="I6" s="18" t="s">
         <v>171</v>
       </c>
-      <c r="F6" s="18" t="s">
+      <c r="J6" s="18" t="s">
         <v>172</v>
       </c>
-      <c r="G6" s="18" t="s">
+      <c r="K6" s="19" t="s">
         <v>173</v>
       </c>
-      <c r="H6" s="18" t="s">
+      <c r="L6" s="18" t="s">
         <v>174</v>
       </c>
-      <c r="I6" s="18" t="s">
-        <v>175</v>
-      </c>
-      <c r="J6" s="18" t="s">
-        <v>176</v>
-      </c>
-      <c r="K6" s="19" t="s">
-        <v>177</v>
-      </c>
-      <c r="L6" s="18" t="s">
-        <v>178</v>
-      </c>
       <c r="M6" s="18" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="N6" s="20">
         <v>46087</v>
@@ -3694,34 +4049,34 @@
     </row>
     <row r="7" spans="1:15" s="18" customFormat="1" ht="30.75">
       <c r="D7" s="18" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="E7" s="18" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="F7" s="18" t="s">
+        <v>175</v>
+      </c>
+      <c r="G7" s="18" t="s">
+        <v>176</v>
+      </c>
+      <c r="H7" s="18" t="s">
+        <v>177</v>
+      </c>
+      <c r="I7" s="19" t="s">
+        <v>178</v>
+      </c>
+      <c r="J7" s="19" t="s">
         <v>179</v>
       </c>
-      <c r="G7" s="18" t="s">
+      <c r="K7" s="19" t="s">
         <v>180</v>
       </c>
-      <c r="H7" s="18" t="s">
-        <v>181</v>
-      </c>
-      <c r="I7" s="19" t="s">
-        <v>182</v>
-      </c>
-      <c r="J7" s="19" t="s">
-        <v>183</v>
-      </c>
-      <c r="K7" s="19" t="s">
-        <v>184</v>
-      </c>
       <c r="L7" s="18" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="M7" s="18" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="N7" s="20">
         <v>46175</v>
@@ -3729,57 +4084,57 @@
     </row>
     <row r="8" spans="1:15" s="18" customFormat="1">
       <c r="D8" s="18" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="E8" s="18" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="F8" s="18" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="G8" s="18" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="H8" s="18" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="I8" s="18" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="K8" s="19"/>
       <c r="N8" s="20"/>
     </row>
     <row r="9" spans="1:15" s="18" customFormat="1">
       <c r="D9" s="18" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="E9" s="18" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="F9" s="18" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="G9" s="18" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
       <c r="H9" s="18" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="I9" s="18" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="K9" s="19"/>
       <c r="N9" s="20"/>
     </row>
     <row r="10" spans="1:15" s="18" customFormat="1" ht="30.75">
       <c r="D10" s="18" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="E10" s="19" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="F10" s="18" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="H10" s="21"/>
       <c r="K10" s="19"/>
@@ -3788,10 +4143,10 @@
     <row r="11" spans="1:15" s="18" customFormat="1" ht="30.75">
       <c r="D11" s="21"/>
       <c r="E11" s="19" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="F11" s="18" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="H11" s="21"/>
       <c r="K11" s="19"/>
@@ -3800,10 +4155,10 @@
     <row r="12" spans="1:15" s="18" customFormat="1" ht="30.75">
       <c r="D12" s="21"/>
       <c r="E12" s="19" t="s">
-        <v>195</v>
+        <v>191</v>
       </c>
       <c r="F12" s="19" t="s">
-        <v>196</v>
+        <v>192</v>
       </c>
       <c r="H12" s="21"/>
       <c r="K12" s="19"/>
@@ -3812,10 +4167,10 @@
     <row r="13" spans="1:15" s="18" customFormat="1" ht="30.75">
       <c r="D13" s="21"/>
       <c r="E13" s="19" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="F13" s="19" t="s">
-        <v>196</v>
+        <v>192</v>
       </c>
       <c r="H13" s="21"/>
       <c r="K13" s="19"/>
@@ -3823,13 +4178,13 @@
     </row>
     <row r="14" spans="1:15" s="18" customFormat="1" ht="30.75">
       <c r="D14" s="24" t="s">
-        <v>160</v>
+        <v>108</v>
       </c>
       <c r="E14" s="19" t="s">
-        <v>93</v>
+        <v>110</v>
       </c>
       <c r="F14" s="19" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
       <c r="K14" s="19"/>
       <c r="N14" s="20"/>
@@ -3887,7 +4242,7 @@
     <row r="28" spans="3:14">
       <c r="E28" s="8"/>
       <c r="H28" s="8"/>
-      <c r="J28" s="52"/>
+      <c r="J28" s="68"/>
     </row>
     <row r="29" spans="3:14">
       <c r="J29" s="8"/>
@@ -3960,17 +4315,17 @@
         <v>2</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
     </row>
     <row r="2" spans="1:14">
-      <c r="B2" s="42" t="s">
-        <v>200</v>
+      <c r="B2" s="39" t="s">
+        <v>196</v>
       </c>
     </row>
     <row r="3" spans="1:14">
-      <c r="B3" s="32" t="s">
-        <v>201</v>
+      <c r="B3" s="31" t="s">
+        <v>197</v>
       </c>
       <c r="N3" s="4"/>
     </row>
@@ -3983,7 +4338,7 @@
     </row>
     <row r="6" spans="1:14">
       <c r="B6" s="2" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
       <c r="N6" s="4"/>
     </row>
@@ -3993,7 +4348,7 @@
         <v>#12</v>
       </c>
       <c r="C7" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
       <c r="N7" s="4"/>
     </row>
@@ -4001,117 +4356,117 @@
       <c r="N8" s="4"/>
     </row>
     <row r="10" spans="1:14" ht="18">
-      <c r="B10" s="28" t="s">
+      <c r="B10" s="27" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14">
+      <c r="B11" s="29" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14">
+      <c r="B12" s="28" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14">
+      <c r="B13" s="28" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14">
+      <c r="B14" s="28" t="s">
         <v>204</v>
-      </c>
-    </row>
-    <row r="11" spans="1:14">
-      <c r="B11" s="30" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="12" spans="1:14">
-      <c r="B12" s="29" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="13" spans="1:14">
-      <c r="B13" s="29" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="14" spans="1:14">
-      <c r="B14" s="29" t="s">
-        <v>208</v>
       </c>
     </row>
     <row r="15" spans="1:14">
       <c r="B15" s="3"/>
     </row>
     <row r="16" spans="1:14">
-      <c r="B16" s="31" t="s">
-        <v>209</v>
+      <c r="B16" s="30" t="s">
+        <v>205</v>
       </c>
     </row>
     <row r="17" spans="2:3">
-      <c r="B17" s="29" t="s">
-        <v>210</v>
+      <c r="B17" s="28" t="s">
+        <v>206</v>
       </c>
     </row>
     <row r="18" spans="2:3">
-      <c r="B18" s="31" t="s">
-        <v>211</v>
+      <c r="B18" s="30" t="s">
+        <v>207</v>
       </c>
     </row>
     <row r="20" spans="2:3">
       <c r="B20" s="5" t="s">
-        <v>212</v>
+        <v>208</v>
       </c>
     </row>
     <row r="21" spans="2:3">
-      <c r="B21" s="32" t="s">
-        <v>213</v>
+      <c r="B21" s="31" t="s">
+        <v>209</v>
       </c>
     </row>
     <row r="22" spans="2:3">
-      <c r="B22" s="32" t="s">
-        <v>214</v>
+      <c r="B22" s="31" t="s">
+        <v>210</v>
       </c>
     </row>
     <row r="23" spans="2:3">
       <c r="B23" s="1"/>
     </row>
     <row r="24" spans="2:3">
-      <c r="B24" s="29" t="s">
-        <v>215</v>
+      <c r="B24" s="28" t="s">
+        <v>211</v>
       </c>
     </row>
     <row r="25" spans="2:3">
       <c r="B25" s="5" t="s">
-        <v>216</v>
-      </c>
-      <c r="C25" s="33" t="s">
-        <v>217</v>
+        <v>212</v>
+      </c>
+      <c r="C25" s="32" t="s">
+        <v>213</v>
       </c>
     </row>
     <row r="26" spans="2:3">
       <c r="B26" t="s">
-        <v>218</v>
+        <v>214</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>219</v>
+        <v>215</v>
       </c>
     </row>
     <row r="27" spans="2:3">
       <c r="B27" t="s">
-        <v>220</v>
+        <v>216</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>221</v>
+        <v>217</v>
       </c>
     </row>
     <row r="28" spans="2:3">
       <c r="B28" t="s">
-        <v>222</v>
+        <v>218</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>223</v>
+        <v>219</v>
       </c>
     </row>
     <row r="29" spans="2:3">
       <c r="B29" t="s">
-        <v>224</v>
+        <v>220</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>225</v>
+        <v>221</v>
       </c>
     </row>
     <row r="30" spans="2:3">
       <c r="B30" t="s">
-        <v>226</v>
+        <v>222</v>
       </c>
       <c r="C30" s="3" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
     </row>
     <row r="31" spans="2:3">
@@ -4119,81 +4474,81 @@
       <c r="C31" s="1"/>
     </row>
     <row r="32" spans="2:3">
-      <c r="B32" s="41" t="s">
-        <v>228</v>
+      <c r="B32" s="38" t="s">
+        <v>224</v>
       </c>
       <c r="C32" s="1"/>
     </row>
     <row r="33" spans="2:3">
       <c r="B33" s="3" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
       <c r="C33" s="1"/>
     </row>
     <row r="34" spans="2:3" ht="21">
-      <c r="B34" s="35" t="s">
-        <v>230</v>
+      <c r="B34" s="34" t="s">
+        <v>226</v>
       </c>
       <c r="C34" s="1"/>
     </row>
     <row r="35" spans="2:3" ht="18.75">
-      <c r="B35" s="40" t="s">
-        <v>231</v>
+      <c r="B35" s="37" t="s">
+        <v>227</v>
       </c>
       <c r="C35" s="1"/>
     </row>
     <row r="36" spans="2:3">
-      <c r="B36" s="34"/>
+      <c r="B36" s="33"/>
       <c r="C36" s="3"/>
     </row>
     <row r="37" spans="2:3">
       <c r="B37" s="11" t="s">
-        <v>232</v>
+        <v>228</v>
       </c>
     </row>
     <row r="38" spans="2:3">
       <c r="B38" s="11" t="s">
-        <v>233</v>
+        <v>229</v>
       </c>
     </row>
     <row r="40" spans="2:3">
-      <c r="B40" s="43" t="s">
-        <v>234</v>
+      <c r="B40" s="40" t="s">
+        <v>230</v>
       </c>
     </row>
     <row r="41" spans="2:3" ht="18">
-      <c r="B41" s="28" t="s">
-        <v>235</v>
+      <c r="B41" s="27" t="s">
+        <v>231</v>
       </c>
     </row>
     <row r="42" spans="2:3">
       <c r="B42" s="3" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="43" spans="2:3">
+      <c r="B43" s="28" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="44" spans="2:3">
+      <c r="B44" s="28" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="45" spans="2:3">
+      <c r="B45" s="28" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="46" spans="2:3">
+      <c r="B46" s="28" t="s">
         <v>236</v>
       </c>
     </row>
-    <row r="43" spans="2:3">
-      <c r="B43" s="29" t="s">
+    <row r="47" spans="2:3">
+      <c r="B47" s="28" t="s">
         <v>237</v>
-      </c>
-    </row>
-    <row r="44" spans="2:3">
-      <c r="B44" s="29" t="s">
-        <v>238</v>
-      </c>
-    </row>
-    <row r="45" spans="2:3">
-      <c r="B45" s="29" t="s">
-        <v>239</v>
-      </c>
-    </row>
-    <row r="46" spans="2:3">
-      <c r="B46" s="29" t="s">
-        <v>240</v>
-      </c>
-    </row>
-    <row r="47" spans="2:3">
-      <c r="B47" s="29" t="s">
-        <v>241</v>
       </c>
     </row>
   </sheetData>
@@ -4204,6 +4559,7 @@
     <hyperlink ref="B6" r:id="rId1" xr:uid="{39ADA6E0-51F0-4485-95AE-61A4DF01666B}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -4217,133 +4573,15 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" t="s">
-        <v>242</v>
+        <v>238</v>
       </c>
     </row>
     <row r="2" spans="1:1" ht="30.75">
       <c r="A2" s="1" t="s">
-        <v>243</v>
+        <v>239</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B4E4155B-D150-4FBC-8164-9A21FFA61D30}">
-  <dimension ref="A2:D5"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="36.5703125" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="2" spans="1:4">
-      <c r="A2" t="s">
-        <v>244</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" ht="60.75">
-      <c r="A3" s="1" t="s">
-        <v>246</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>247</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" ht="30.75">
-      <c r="A4" s="1" t="s">
-        <v>248</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4">
-      <c r="A5" s="1" t="s">
-        <v>250</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D3C8E892-55D5-4419-AE3A-0965C50FB74C}">
-  <dimension ref="A1:C34"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="36.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="2.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="19.42578125" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:1">
-      <c r="A1" t="s">
-        <v>251</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1" ht="60.75">
-      <c r="A2" s="1" t="s">
-        <v>252</v>
-      </c>
-    </row>
-    <row r="3" spans="1:1">
-      <c r="A3" s="3" t="s">
-        <v>253</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3">
-      <c r="A27" t="s">
-        <v>254</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" ht="57">
-      <c r="A29" s="48" t="s">
-        <v>255</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3">
-      <c r="A30" s="3" t="s">
-        <v>256</v>
-      </c>
-      <c r="B30" s="49" t="s">
-        <v>257</v>
-      </c>
-      <c r="C30" s="50" t="s">
-        <v>258</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3">
-      <c r="A31" s="29" t="s">
-        <v>259</v>
-      </c>
-      <c r="B31" s="3"/>
-      <c r="C31" s="3"/>
-    </row>
-    <row r="32" spans="1:3">
-      <c r="A32" s="3" t="s">
-        <v>260</v>
-      </c>
-      <c r="B32" s="49" t="s">
-        <v>257</v>
-      </c>
-      <c r="C32" s="50" t="s">
-        <v>261</v>
-      </c>
-    </row>
-    <row r="34" spans="1:1" ht="30.75">
-      <c r="A34" s="51" t="s">
-        <v>262</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
-</worksheet>
 </file>
</xml_diff>